<commit_message>
fix: update demo xlsx headers to match v2.2.6 column spec
Add missing front_card_reading column to all 3 demo files.
Headers now follow the full 7-column order:
front_card, front_card_reading, back_card_meaning, back_card_sentence,
back_card_sentence_meaning, back_card_opposite, back_card_opposite_meaning

Also refactor create_demo.py to use shared HEADERS/COL_WIDTHS constants
so all demo files stay in sync automatically.
</commit_message>
<xml_diff>
--- a/how_to_use/demo_korean.xlsx
+++ b/how_to_use/demo_korean.xlsx
@@ -413,15 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -432,25 +433,30 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>front_card_reading</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>back_card_meaning</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>back_card_sentence</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>back_card_sentence_meaning</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>back_card_opposite</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>back_card_opposite_meaning</t>
         </is>
@@ -467,6 +473,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -479,6 +486,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -491,6 +499,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -503,6 +512,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -515,6 +525,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>